<commit_message>
feat: add financing options widget with live scenario recalculation
</commit_message>
<xml_diff>
--- a/examples/zips/92258/92258_for_sale.xlsx
+++ b/examples/zips/92258/92258_for_sale.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR5"/>
+  <dimension ref="A1:AR4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -721,7 +721,7 @@
         <v>1960</v>
       </c>
       <c r="R2" t="n">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="S2" t="inlineStr">
         <is>
@@ -750,12 +750,12 @@
       </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>Incredible investment Opportunity in this unique property with Two homes on a spacious 8,712 sq ft lot located in North Palm Springs. Complete with Beautiful views of the snow capped San Jacinto Mountains!! Since this is the First time this property has been on the market in 35 years, it offers an excellent potential for renovation and investment as a fix and flip project, live in one and rent the other, or create the perfect multi-generational environment. The main home has 2 bedrooms and 1 bath. Kitchen is open to the family room. 2nd exterior door provides quick access to the garage. The second home has 1 bedroom and 1 bath. Total square footage is 1,880 sq ft per assessor office and buyer to verify permits. Conveniently located one-car garage between the 2 homes. The workshop is the perfect area to transform it into a home office, children's play area, gym, game room, an outdoor lounge.... The possibilities are endless!! Newer cemented driveway. Relax and take in the mountain views under the vinyl courtyard patio. The side yard is a blank canvas for your creativity. There is damage to the ceiling in the second home and dried mud on the floor of the workshop. Just bring your tools and let the renovations begin!!</t>
+          <t>Incredible investment Opportunity in this unique property with Two homes on a spacious 8,712 sq ft lot located in North Palm Springs. Complete with Beautiful views of the San Jacinto Mountains!! Since this is the First time this property has been on the market in 35 years, it offers an excellent potential for renovation and investment as a fix and flip project, live in one and rent the other, or create the perfect multi-generational environment. The main home has 2 bedrooms and 1 bath. Kitchen is open to the family room. 2nd exterior door provides quick access to the garage. The second home has 1 bedroom and 1 bath. Total square footage is 1,880 sq ft per assessor office and buyer to verify permits. Conveniently located one-car garage between the 2 homes. Each home has its own electric meter and water heater. The workshop is the perfect area to transform it into a home office, children's play area, gym, game room, an outdoor lounge.... The possibilities are endless!! Newer cemented driveway. Relax and take in the mountain views under the shady vinyl courtyard patio. The side yard is a blank canvas for your creativity. There is damage to one area of the ceiling in the second home and dried mud on the floor of the workshop. Just bring your tools and let the renovations begin!!</t>
         </is>
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>Incredible investment Opportunity in this unique property with Two homes on a spacious 8,712 sq ft lot located in North Palm Springs. Complete with Beautiful views of the snow capped San Jacinto Mountains!! Since this is the First time this property has been on the market in 35 years, it offers an excellent potential for renovation and investment as a fix and flip project, live in one and rent the other, or create the perfect multi-generational environment. The main home has 2 bedrooms and 1 bath. Kitchen is open to the family room. 2nd exterior door provides quick access to the garage. The second home has 1 bedroom and 1 bath. Total square footage is 1,880 sq ft per assessor office and buyer to verify permits. Conveniently located one-car garage between the 2 homes. The workshop is the perfect area to transform it into a home office, children's play area, gym, game room, an outdoor lounge.... The possibilities are endless!! Newer cemented driveway. Relax and take in the mountain views under the vinyl courtyard patio. The side yard is a blank canvas for your creativity. There is damage to the ceiling in the second home and dried mud on the floor of the workshop. Just bring your tools and let the renovations begin!!</t>
+          <t>Incredible investment Opportunity in this unique property with Two homes on a spacious 8,712 sq ft lot located in North Palm Springs. Complete with Beautiful views of the San Jacinto Mountains!! Since this is the First time this property has been on the market in 35 years, it offers an excellent potential for renovation and investment as a fix and flip project, live in one and rent the other, or create the perfect multi-generational environment. The main home has 2 bedrooms and 1 bath. Kitchen is open to the family room. 2nd exterior door provides quick access to the garage. The second home has 1 bedroom and 1 bath. Total square footage is 1,880 sq ft per assessor office and buyer to verify permits. Conveniently located one-car garage between the 2 homes. Each home has its own electric meter and water heater. The workshop is the perfect area to transform it into a home office, children's play area, gym, game room, an outdoor lounge.... The possibilities are endless!! Newer cemented driveway. Relax and take in the mountain views under the shady vinyl courtyard patio. The side yard is a blank canvas for your creativity. There is damage to one area of the ceiling in the second home and dried mud on the floor of the workshop. Just bring your tools and let the renovations begin!!</t>
         </is>
       </c>
       <c r="AB2" t="n">
@@ -776,7 +776,7 @@
       </c>
       <c r="AF2" t="inlineStr">
         <is>
-          <t>[{"href": "https://ap.rdcpix.com/b93b02e1982139086b6613d76e15462fl-m3846321327s.jpg", "labels": ["exterior", "exterior", "exterior", "exterior", "exterior", "exterior"]}, {"href": "https://ap.rdcpix.com/b93b02e1982139086b6613d76e15462fl-m3435647156s.jpg", "labels": ["exterior", "exterior"]}, {"href": "https://ap.rdcpix.com/b93b02e1982139086b6613d76e15462fl-m2348238812s.jpg", "labels": ["exterior", "exterior", "exterior"]}, {"href": "https://ap.rdcpix.com/b93b02e1982139086b6613d76e15462fl-m1053058417s.jpg", "labels": ["exterior", "exterior"]}]</t>
+          <t>[{"href": "https://ap.rdcpix.com/b93b02e1982139086b6613d76e15462fl-m1491716075s.jpg", "labels": ["exterior", "exterior", "exterior", "exterior", "exterior", "exterior"]}, {"href": "https://ap.rdcpix.com/b93b02e1982139086b6613d76e15462fl-m826847626s.jpg", "labels": ["exterior", "exterior"]}, {"href": "https://ap.rdcpix.com/b93b02e1982139086b6613d76e15462fl-m2282386473s.jpg", "labels": ["exterior", "exterior", "exterior"]}, {"href": "https://ap.rdcpix.com/b93b02e1982139086b6613d76e15462fl-m709621985s.jpg", "labels": ["exterior", "exterior"]}, {"href": "https://ap.rdcpix.com/b93b02e1982139086b6613d76e15462fl-m2341698334s.jpg", "labels": ["unknown"]}, {"href": "https://ap.rdcpix.com/b93b02e1982139086b6613d76e15462fl-m3726687476s.jpg", "labels": ["kitchen"]}, {"href": "https://ap.rdcpix.com/b93b02e1982139086b6613d76e15462fl-m179962357s.jpg", "labels": ["unknown"]}, {"href": "https://ap.rdcpix.com/b93b02e1982139086b6613d76e15462fl-m2553722161s.jpg", "labels": ["unknown"]}, {"href": "https://ap.rdcpix.com/b93b02e1982139086b6613d76e15462fl-m3168336684s.jpg", "labels": ["unknown"]}, {"href": "https://ap.rdcpix.com/b93b02e1982139086b6613d76e15462fl-m2838721217s.jpg", "labels": ["exterior", "exterior"]}, {"href": "https://ap.rdcpix.com/b93b02e1982139086b6613d76e15462fl-m1008714397s.jpg", "labels": ["unknown"]}, {"href": "https://ap.rdcpix.com/b93b02e1982139086b6613d76e15462fl-m1440061965s.jpg", "labels": ["unknown"]}, {"href": "https://ap.rdcpix.com/b93b02e1982139086b6613d76e15462fl-m3571219395s.jpg", "labels": ["unknown"]}]</t>
         </is>
       </c>
       <c r="AG2" t="b">
@@ -897,7 +897,7 @@
         <v>1950</v>
       </c>
       <c r="R3" t="n">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="S3" t="inlineStr">
         <is>
@@ -1069,7 +1069,7 @@
         <v>1972</v>
       </c>
       <c r="R4" t="n">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="S4" t="inlineStr">
         <is>
@@ -1165,178 +1165,6 @@
         <v>0</v>
       </c>
       <c r="AR4" t="inlineStr">
-        <is>
-          <t>details,photo_tags,tags</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>https://www.realtor.com/realestateandhomes-detail/61612-Sagebrush-Rd_North-Palm-Springs_CA_92258_M10762-68959</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>1076268959</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>SINGLE_FAMILY</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>FOR_SALE</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>61612 Sagebrush Rd</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>North Palm Springs</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>CA</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>92258</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>Riverside</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="n">
-        <v>33.929266</v>
-      </c>
-      <c r="L5" t="n">
-        <v>-116.587339</v>
-      </c>
-      <c r="M5" t="n">
-        <v>4</v>
-      </c>
-      <c r="N5" t="n">
-        <v>2</v>
-      </c>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="n">
-        <v>1985</v>
-      </c>
-      <c r="Q5" t="n">
-        <v>1958</v>
-      </c>
-      <c r="R5" t="n">
-        <v>267</v>
-      </c>
-      <c r="S5" t="inlineStr">
-        <is>
-          <t>2025-08-02 01:22:52</t>
-        </is>
-      </c>
-      <c r="T5" t="inlineStr">
-        <is>
-          <t>2020-11-23 00:00:00</t>
-        </is>
-      </c>
-      <c r="U5" t="n">
-        <v>550000</v>
-      </c>
-      <c r="V5" t="n">
-        <v>343000</v>
-      </c>
-      <c r="W5" t="n">
-        <v>277.0780856423174</v>
-      </c>
-      <c r="X5" t="n">
-        <v>217800</v>
-      </c>
-      <c r="Y5" t="n">
-        <v>217800</v>
-      </c>
-      <c r="Z5" t="inlineStr">
-        <is>
-          <t>Enjoy the desert tranquility and breathtaking views of San Jacinto from your own private gateway. This unique 4 bedrooms, 2 bath home on a huge 5 acres lot, offers the perfect blend of comfort and convenience. Thoughtfully designed for the perfect escape from the city, this home offers stunning sunsets with mountain views, easy access to outdoor adventure and a sleek, low-maintenance lifestyle. Whether you looking for a weekend retreat or an Airbnb income generator smart investment, this home delivers style, comfort, and convenience. There are so many opportunities offered by this property and its extensive 5 acres of land. For the savvy investor, the Airbnb permits are still available in this neighborhood. Interested in an assumable loan in this high interest rate environment? Seller has an FHA assumable loan at an incredible low rate (subject to seller's current lender approval). Desert Hills Premium Outlets is only 15 minutes away and downtown Palm Springs is 20 minutes away.</t>
-        </is>
-      </c>
-      <c r="AA5" t="inlineStr">
-        <is>
-          <t>Enjoy the desert tranquility and breathtaking views of San Jacinto from your own private gateway. This unique 4 bedrooms, 2 bath home on a huge 5 acres lot, offers the perfect blend of comfort and convenience. Thoughtfully designed for the perfect escape from the city, this home offers stunning sunsets with mountain views, easy access to outdoor adventure and a sleek, low-maintenance lifestyle. Whether you looking for a weekend retreat or an Airbnb income generator smart investment, this home delivers style, comfort, and convenience. There are so many opportunities offered by this property and its extensive 5 acres of land. For the savvy investor, the Airbnb permits are still available in this neighborhood. Interested in an assumable loan in this high interest rate environment? Seller has an FHA assumable loan at an incredible low rate (subject to seller's current lender approval). Desert Hills Premium Outlets is only 15 minutes away and downtown Palm Springs is 20 minutes away.</t>
-        </is>
-      </c>
-      <c r="AB5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD5" t="inlineStr">
-        <is>
-          <t>[{"category": "Bedrooms", "text": ["Bedrooms: 4", "Bedrooms On Main Level: 4"], "parent_category": "Interior"}, {"category": "Bathrooms", "text": ["Total Bathrooms: 2", "Full Bathrooms: 2", "Bathrooms On Main Level: 2"], "parent_category": "Interior"}, {"category": "Other Rooms", "text": ["All Bedrooms Down"], "parent_category": "Interior"}, {"category": "Appliances", "text": ["Laundry Features: Inside"], "parent_category": "Interior"}, {"category": "Heating and Cooling", "text": ["Cooling Features: Central Air", "Fireplace Features: Living Room", "Heating Features: Central", "Heating: Yes"], "parent_category": "Interior"}, {"category": "Kitchen and Dining", "text": ["Breakfast Room Description: In Kitchen"], "parent_category": "Interior"}, {"category": "Land Info", "text": ["Additional Parcels: No", "Land Lease: No", "Lot Description: 2-5 Units/Acre", "Lot Size Acres: 5.0", "Lot Size Source: Assessor", "Lot Size Square Feet: 217800"], "parent_category": "Exterior"}, {"category": "Exterior and Lot Features", "text": ["Road Surface Type: Unpaved"], "parent_category": "Exterior"}, {"category": "Garage and Parking", "text": ["Parking Features: Carport"], "parent_category": "Exterior"}, {"category": "Home Features", "text": ["View: Desert, Mountain(s)"], "parent_category": "Exterior"}, {"category": "Homeowners Association", "text": ["Association: No", "Calculated Total Monthly Association Fees: 0"], "parent_category": "Community"}, {"category": "Multi-Unit Info", "text": ["Number of Units: 1"], "parent_category": "Community"}, {"category": "School Information", "text": ["School District: Palm Springs Unified"], "parent_category": "Community"}, {"category": "Rental Info", "text": ["Lease Considered: No"], "parent_category": "Community"}, {"category": "Amenities and Community Features", "text": ["Community Features: Hiking, Mountainous, Rural"], "parent_category": "Community"}, {"category": "Other Property Info", "text": ["Source Listing Status: Active", "County: Riverside", "Directions: Indian Canyon Dr to Dillon Rd, right on Valley View Dr, right on Sagebrush Rd (2nd street).", "Source Property Type: Residential", "Area: 699 - Not Defined", "Source Neighborhood: 699 - Not Defined", "Parcel Number: 668220014", "Postal Code Plus 4: 0496", "Zoning: W-2", "Property Subtype: Single Family Residence"], "parent_category": "Listing"}, {"category": "Building and Construction", "text": ["Total Square Feet Living: 1985.00", "Year Built: 1958", "Common Walls: No Common Walls", "Entry Level: 1", "Entry Location: main", "Levels: One", "Living Area Source: Assessor", "Living Area Units: Square Feet", "Property Age: 68", "Property Attached: No", "Property Condition: Turnkey", "Levels or Stories: One", "Building Total Stories: 1", "Structure Type: House", "Elevation Units: Feet", "Year Built Source: Assessor", "Architectural Style: Ranch"], "parent_category": "Features"}, {"category": "Utilities", "text": ["Sewer: Septic Type Unknown", "Water Source: Public"], "parent_category": "Features"}]</t>
-        </is>
-      </c>
-      <c r="AE5" t="inlineStr">
-        <is>
-          <t>["carport", "central_air", "central_heat", "fireplace", "hill_or_mountain_view", "laundry_room", "view", "single_story", "rental_property", "big_lot", "mountain_view", "breathtaking_views", "views"]</t>
-        </is>
-      </c>
-      <c r="AF5" t="inlineStr">
-        <is>
-          <t>[{"href": "https://ap.rdcpix.com/42f13f44dc366a51b18f9200aa2a88eel-m3200075157s.jpg", "labels": ["exterior", "exterior", "exterior"]}, {"href": "https://ap.rdcpix.com/42f13f44dc366a51b18f9200aa2a88eel-m1664683402s.jpg", "labels": ["exterior", "exterior", "exterior", "exterior"]}, {"href": "https://ap.rdcpix.com/42f13f44dc366a51b18f9200aa2a88eel-m46284255s.jpg", "labels": ["exterior", "exterior"]}, {"href": "https://ap.rdcpix.com/42f13f44dc366a51b18f9200aa2a88eel-m1575544242s.jpg", "labels": ["exterior", "exterior", "exterior"]}, {"href": "https://ap.rdcpix.com/42f13f44dc366a51b18f9200aa2a88eel-m1372693044s.jpg", "labels": ["living_room"]}, {"href": "https://ap.rdcpix.com/42f13f44dc366a51b18f9200aa2a88eel-m2065356000s.jpg", "labels": ["unknown"]}, {"href": "https://ap.rdcpix.com/42f13f44dc366a51b18f9200aa2a88eel-m2622041543s.jpg", "labels": ["living_room"]}, {"href": "https://ap.rdcpix.com/42f13f44dc366a51b18f9200aa2a88eel-m2916504500s.jpg", "labels": ["living_room"]}, {"href": "https://ap.rdcpix.com/42f13f44dc366a51b18f9200aa2a88eel-m1923579425s.jpg", "labels": ["living_room"]}, {"href": "https://ap.rdcpix.com/42f13f44dc366a51b18f9200aa2a88eel-m2504931907s.jpg", "labels": ["living_room"]}, {"href": "https://ap.rdcpix.com/42f13f44dc366a51b18f9200aa2a88eel-m2014307786s.jpg", "labels": ["unknown"]}, {"href": "https://ap.rdcpix.com/42f13f44dc366a51b18f9200aa2a88eel-m781359343s.jpg", "labels": ["kitchen"]}, {"href": "https://ap.rdcpix.com/42f13f44dc366a51b18f9200aa2a88eel-m267476246s.jpg", "labels": ["kitchen"]}, {"href": "https://ap.rdcpix.com/42f13f44dc366a51b18f9200aa2a88eel-m1464024972s.jpg", "labels": ["kitchen"]}, {"href": "https://ap.rdcpix.com/42f13f44dc366a51b18f9200aa2a88eel-m1534993186s.jpg", "labels": ["kitchen"]}, {"href": "https://ap.rdcpix.com/42f13f44dc366a51b18f9200aa2a88eel-m2629666874s.jpg", "labels": ["bedroom"]}, {"href": "https://ap.rdcpix.com/42f13f44dc366a51b18f9200aa2a88eel-m3073786309s.jpg", "labels": ["bedroom"]}, {"href": "https://ap.rdcpix.com/42f13f44dc366a51b18f9200aa2a88eel-m703726341s.jpg", "labels": ["unknown"]}, {"href": "https://ap.rdcpix.com/42f13f44dc366a51b18f9200aa2a88eel-m1126583630s.jpg", "labels": ["bedroom"]}, {"href": "https://ap.rdcpix.com/42f13f44dc366a51b18f9200aa2a88eel-m722501013s.jpg", "labels": ["living_room"]}, {"href": "https://ap.rdcpix.com/42f13f44dc366a51b18f9200aa2a88eel-m2508561337s.jpg", "labels": ["bedroom"]}, {"href": "https://ap.rdcpix.com/42f13f44dc366a51b18f9200aa2a88eel-m2589039701s.jpg", "labels": ["unknown"]}, {"href": "https://ap.rdcpix.com/42f13f44dc366a51b18f9200aa2a88eel-m172142027s.jpg", "labels": ["living_room"]}, {"href": "https://ap.rdcpix.com/42f13f44dc366a51b18f9200aa2a88eel-m3296881792s.jpg", "labels": ["exterior", "exterior", "exterior"]}, {"href": "https://ap.rdcpix.com/42f13f44dc366a51b18f9200aa2a88eel-m562999200s.jpg", "labels": ["bathroom"]}, {"href": "https://ap.rdcpix.com/42f13f44dc366a51b18f9200aa2a88eel-m4170372171s.jpg", "labels": ["bathroom"]}, {"href": "https://ap.rdcpix.com/42f13f44dc366a51b18f9200aa2a88eel-m1410007878s.jpg", "labels": ["bathroom"]}, {"href": "https://ap.rdcpix.com/42f13f44dc366a51b18f9200aa2a88eel-m2981440721s.jpg", "labels": ["bathroom"]}, {"href": "https://ap.rdcpix.com/42f13f44dc366a51b18f9200aa2a88eel-m1983704122s.jpg", "labels": ["exterior", "exterior", "exterior"]}, {"href": "https://ap.rdcpix.com/42f13f44dc366a51b18f9200aa2a88eel-m224018912s.jpg", "labels": ["exterior"]}, {"href": "https://ap.rdcpix.com/42f13f44dc366a51b18f9200aa2a88eel-m3639343553s.jpg", "labels": ["exterior", "exterior", "exterior", "swimming_pool"]}, {"href": "https://ap.rdcpix.com/42f13f44dc366a51b18f9200aa2a88eel-m2637726737s.jpg", "labels": ["exterior", "exterior", "exterior"]}, {"href": "https://ap.rdcpix.com/42f13f44dc366a51b18f9200aa2a88eel-m3581863079s.jpg", "labels": ["exterior", "exterior", "exterior"]}, {"href": "https://ap.rdcpix.com/42f13f44dc366a51b18f9200aa2a88eel-m3098624546s.jpg", "labels": ["exterior", "exterior"]}, {"href": "https://ap.rdcpix.com/42f13f44dc366a51b18f9200aa2a88eel-m3621514268s.jpg", "labels": ["exterior", "exterior", "exterior"]}, {"href": "https://ap.rdcpix.com/42f13f44dc366a51b18f9200aa2a88eel-m1553673971s.jpg", "labels": ["exterior", "exterior", "exterior"]}, {"href": "https://ap.rdcpix.com/42f13f44dc366a51b18f9200aa2a88eel-m1693713241s.jpg", "labels": ["exterior"]}, {"href": "https://ap.rdcpix.com/42f13f44dc366a51b18f9200aa2a88eel-m3787841785s.jpg", "labels": ["exterior"]}, {"href": "https://ap.rdcpix.com/42f13f44dc366a51b18f9200aa2a88eel-m4249936533s.jpg", "labels": ["exterior", "exterior"]}, {"href": "https://ap.rdcpix.com/42f13f44dc366a51b18f9200aa2a88eel-m291358948s.jpg", "labels": ["exterior"]}]</t>
-        </is>
-      </c>
-      <c r="AG5" t="b">
-        <v>1</v>
-      </c>
-      <c r="AH5" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="AI5" t="b">
-        <v>0</v>
-      </c>
-      <c r="AJ5" t="b">
-        <v>0</v>
-      </c>
-      <c r="AK5" t="b">
-        <v>0</v>
-      </c>
-      <c r="AL5" t="b">
-        <v>0</v>
-      </c>
-      <c r="AM5" t="b">
-        <v>0</v>
-      </c>
-      <c r="AN5" t="inlineStr">
-        <is>
-          <t>low</t>
-        </is>
-      </c>
-      <c r="AO5" t="inlineStr">
-        <is>
-          <t>details,photo_tags,tags</t>
-        </is>
-      </c>
-      <c r="AP5" t="inlineStr">
-        <is>
-          <t>swimming pool</t>
-        </is>
-      </c>
-      <c r="AQ5" t="b">
-        <v>1</v>
-      </c>
-      <c r="AR5" t="inlineStr">
         <is>
           <t>details,photo_tags,tags</t>
         </is>

</xml_diff>